<commit_message>
Replace 154 Partners demo branding with NL Intelligence
</commit_message>
<xml_diff>
--- a/demo_assets/reports/Tallis_Brook_Accounting_Sep2026_MonthlyReview.xlsx
+++ b/demo_assets/reports/Tallis_Brook_Accounting_Sep2026_MonthlyReview.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Financial Performance" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Findings" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Source Evidence" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Data Quality" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Extracted Detail" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Exceptions" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Analyst Execution" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Statement Evidence" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Executive Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Financial Performance" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Evidence" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Extracted Detail" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exceptions" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Analyst Execution" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statement Evidence" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'Executive Summary'!$A$1:$L$67</definedName>
@@ -1470,7 +1470,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="49" t="inlineStr">
         <is>
-          <t>154 Partners · Portfolio Reporting Copilot · Product Demo · Synthetic Data</t>
+          <t>NL Intelligence · Portfolio Reporting Copilot · Product Demo · Synthetic Data</t>
         </is>
       </c>
     </row>
@@ -65745,7 +65745,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="49" t="inlineStr">
         <is>
-          <t>154 Partners · Portfolio Reporting Copilot · Product Demo · Synthetic Data</t>
+          <t>NL Intelligence · Portfolio Reporting Copilot · Product Demo · Synthetic Data</t>
         </is>
       </c>
     </row>

</xml_diff>